<commit_message>
chore: checkpoint before charge state dropdown update
</commit_message>
<xml_diff>
--- a/docs/reference/电龙AI行为记录模板Excel.xlsx
+++ b/docs/reference/电龙AI行为记录模板Excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/miko/Code/web-behavior-tree/docs/reference/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F86E946B-0653-1342-9DFD-1F6A0D0F9038}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{558BE33C-5D5B-3C4D-BE88-E13E2A337734}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30740" yWindow="600" windowWidth="15340" windowHeight="23820" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4000" yWindow="6140" windowWidth="16900" windowHeight="23820" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="导出摘要" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="下拉选项" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">行为记录模板!$A$1:$A$200</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">行为记录模板!$A$1:$D$76</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
@@ -2033,6 +2033,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:E200"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="1"/>
   <cols>
@@ -2059,7 +2060,7 @@
       </c>
       <c r="E1" s="7"/>
     </row>
-    <row r="2" spans="1:5" ht="19" customHeight="1">
+    <row r="2" spans="1:5" ht="19" hidden="1" customHeight="1">
       <c r="A2" s="8" t="s">
         <v>10</v>
       </c>
@@ -2072,7 +2073,7 @@
       <c r="D2" s="10"/>
       <c r="E2" s="11"/>
     </row>
-    <row r="3" spans="1:5" ht="19" customHeight="1">
+    <row r="3" spans="1:5" ht="19" hidden="1" customHeight="1">
       <c r="A3" s="8" t="s">
         <v>10</v>
       </c>
@@ -2085,7 +2086,7 @@
       <c r="D3" s="10"/>
       <c r="E3" s="11"/>
     </row>
-    <row r="4" spans="1:5" ht="24" customHeight="1">
+    <row r="4" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A4" s="8" t="s">
         <v>10</v>
       </c>
@@ -2098,7 +2099,7 @@
       <c r="D4" s="10"/>
       <c r="E4" s="11"/>
     </row>
-    <row r="5" spans="1:5" ht="24" customHeight="1">
+    <row r="5" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A5" s="8" t="s">
         <v>14</v>
       </c>
@@ -2111,7 +2112,7 @@
       <c r="D5" s="10"/>
       <c r="E5" s="11"/>
     </row>
-    <row r="6" spans="1:5" ht="24" customHeight="1">
+    <row r="6" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A6" s="8" t="s">
         <v>10</v>
       </c>
@@ -2124,7 +2125,7 @@
       <c r="D6" s="10"/>
       <c r="E6" s="11"/>
     </row>
-    <row r="7" spans="1:5" ht="24" customHeight="1">
+    <row r="7" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A7" s="8" t="s">
         <v>10</v>
       </c>
@@ -2137,7 +2138,7 @@
       <c r="D7" s="10"/>
       <c r="E7" s="11"/>
     </row>
-    <row r="8" spans="1:5" ht="24" customHeight="1">
+    <row r="8" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A8" s="8" t="s">
         <v>14</v>
       </c>
@@ -2150,7 +2151,7 @@
       <c r="D8" s="10"/>
       <c r="E8" s="11"/>
     </row>
-    <row r="9" spans="1:5" ht="24" customHeight="1">
+    <row r="9" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A9" s="8" t="s">
         <v>19</v>
       </c>
@@ -2163,7 +2164,7 @@
       <c r="D9" s="10"/>
       <c r="E9" s="11"/>
     </row>
-    <row r="10" spans="1:5" ht="24" customHeight="1">
+    <row r="10" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A10" s="8" t="s">
         <v>10</v>
       </c>
@@ -2176,7 +2177,7 @@
       <c r="D10" s="10"/>
       <c r="E10" s="11"/>
     </row>
-    <row r="11" spans="1:5" ht="24" customHeight="1">
+    <row r="11" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A11" s="8" t="s">
         <v>10</v>
       </c>
@@ -2189,7 +2190,7 @@
       <c r="D11" s="10"/>
       <c r="E11" s="11"/>
     </row>
-    <row r="12" spans="1:5" ht="24" customHeight="1">
+    <row r="12" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A12" s="8" t="s">
         <v>14</v>
       </c>
@@ -2202,7 +2203,7 @@
       <c r="D12" s="10"/>
       <c r="E12" s="11"/>
     </row>
-    <row r="13" spans="1:5" ht="24" customHeight="1">
+    <row r="13" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A13" s="8" t="s">
         <v>14</v>
       </c>
@@ -2215,7 +2216,7 @@
       <c r="D13" s="10"/>
       <c r="E13" s="11"/>
     </row>
-    <row r="14" spans="1:5" ht="24" customHeight="1">
+    <row r="14" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A14" s="8" t="s">
         <v>10</v>
       </c>
@@ -2228,7 +2229,7 @@
       <c r="D14" s="10"/>
       <c r="E14" s="11"/>
     </row>
-    <row r="15" spans="1:5" ht="24" customHeight="1">
+    <row r="15" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A15" s="8" t="s">
         <v>10</v>
       </c>
@@ -2241,7 +2242,7 @@
       <c r="D15" s="10"/>
       <c r="E15" s="11"/>
     </row>
-    <row r="16" spans="1:5" ht="24" customHeight="1">
+    <row r="16" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A16" s="8" t="s">
         <v>14</v>
       </c>
@@ -2254,7 +2255,7 @@
       <c r="D16" s="10"/>
       <c r="E16" s="11"/>
     </row>
-    <row r="17" spans="1:5" ht="24" customHeight="1">
+    <row r="17" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A17" s="8" t="s">
         <v>10</v>
       </c>
@@ -2267,7 +2268,7 @@
       <c r="D17" s="10"/>
       <c r="E17" s="11"/>
     </row>
-    <row r="18" spans="1:5" ht="24" customHeight="1">
+    <row r="18" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A18" s="8" t="s">
         <v>10</v>
       </c>
@@ -2280,7 +2281,7 @@
       <c r="D18" s="10"/>
       <c r="E18" s="11"/>
     </row>
-    <row r="19" spans="1:5" ht="24" customHeight="1">
+    <row r="19" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A19" s="8" t="s">
         <v>14</v>
       </c>
@@ -2293,7 +2294,7 @@
       <c r="D19" s="10"/>
       <c r="E19" s="11"/>
     </row>
-    <row r="20" spans="1:5" ht="24" customHeight="1">
+    <row r="20" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A20" s="8" t="s">
         <v>14</v>
       </c>
@@ -2306,7 +2307,7 @@
       <c r="D20" s="10"/>
       <c r="E20" s="11"/>
     </row>
-    <row r="21" spans="1:5" ht="24" customHeight="1">
+    <row r="21" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A21" s="8" t="s">
         <v>14</v>
       </c>
@@ -2319,7 +2320,7 @@
       <c r="D21" s="10"/>
       <c r="E21" s="11"/>
     </row>
-    <row r="22" spans="1:5" ht="24" customHeight="1">
+    <row r="22" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A22" s="8" t="s">
         <v>19</v>
       </c>
@@ -2332,7 +2333,7 @@
       <c r="D22" s="10"/>
       <c r="E22" s="11"/>
     </row>
-    <row r="23" spans="1:5" ht="24" customHeight="1">
+    <row r="23" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A23" s="8" t="s">
         <v>14</v>
       </c>
@@ -2345,7 +2346,7 @@
       <c r="D23" s="10"/>
       <c r="E23" s="11"/>
     </row>
-    <row r="24" spans="1:5" ht="24" customHeight="1">
+    <row r="24" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A24" s="8" t="s">
         <v>14</v>
       </c>
@@ -2358,7 +2359,7 @@
       <c r="D24" s="10"/>
       <c r="E24" s="11"/>
     </row>
-    <row r="25" spans="1:5" ht="24" customHeight="1">
+    <row r="25" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A25" s="8" t="s">
         <v>10</v>
       </c>
@@ -2371,7 +2372,7 @@
       <c r="D25" s="10"/>
       <c r="E25" s="11"/>
     </row>
-    <row r="26" spans="1:5" ht="24" customHeight="1">
+    <row r="26" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A26" s="8" t="s">
         <v>14</v>
       </c>
@@ -2384,7 +2385,7 @@
       <c r="D26" s="10"/>
       <c r="E26" s="11"/>
     </row>
-    <row r="27" spans="1:5" ht="24" customHeight="1">
+    <row r="27" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A27" s="8" t="s">
         <v>10</v>
       </c>
@@ -2397,7 +2398,7 @@
       <c r="D27" s="10"/>
       <c r="E27" s="11"/>
     </row>
-    <row r="28" spans="1:5" ht="24" customHeight="1">
+    <row r="28" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A28" s="8" t="s">
         <v>14</v>
       </c>
@@ -2410,7 +2411,7 @@
       <c r="D28" s="10"/>
       <c r="E28" s="11"/>
     </row>
-    <row r="29" spans="1:5" ht="24" customHeight="1">
+    <row r="29" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A29" s="8" t="s">
         <v>10</v>
       </c>
@@ -2423,7 +2424,7 @@
       <c r="D29" s="10"/>
       <c r="E29" s="11"/>
     </row>
-    <row r="30" spans="1:5" ht="24" customHeight="1">
+    <row r="30" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A30" s="8" t="s">
         <v>10</v>
       </c>
@@ -2436,7 +2437,7 @@
       <c r="D30" s="10"/>
       <c r="E30" s="11"/>
     </row>
-    <row r="31" spans="1:5" ht="24" customHeight="1">
+    <row r="31" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A31" s="8" t="s">
         <v>10</v>
       </c>
@@ -2449,7 +2450,7 @@
       <c r="D31" s="10"/>
       <c r="E31" s="11"/>
     </row>
-    <row r="32" spans="1:5" ht="24" customHeight="1">
+    <row r="32" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A32" s="8" t="s">
         <v>10</v>
       </c>
@@ -2462,7 +2463,7 @@
       <c r="D32" s="10"/>
       <c r="E32" s="11"/>
     </row>
-    <row r="33" spans="1:5" ht="24" customHeight="1">
+    <row r="33" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A33" s="8" t="s">
         <v>10</v>
       </c>
@@ -2475,7 +2476,7 @@
       <c r="D33" s="10"/>
       <c r="E33" s="11"/>
     </row>
-    <row r="34" spans="1:5" ht="24" customHeight="1">
+    <row r="34" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A34" s="8" t="s">
         <v>19</v>
       </c>
@@ -2488,7 +2489,7 @@
       <c r="D34" s="10"/>
       <c r="E34" s="11"/>
     </row>
-    <row r="35" spans="1:5" ht="24" customHeight="1">
+    <row r="35" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A35" s="8" t="s">
         <v>14</v>
       </c>
@@ -2501,7 +2502,7 @@
       <c r="D35" s="10"/>
       <c r="E35" s="11"/>
     </row>
-    <row r="36" spans="1:5" ht="24" customHeight="1">
+    <row r="36" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A36" s="8" t="s">
         <v>10</v>
       </c>
@@ -2514,7 +2515,7 @@
       <c r="D36" s="10"/>
       <c r="E36" s="11"/>
     </row>
-    <row r="37" spans="1:5" ht="24" customHeight="1">
+    <row r="37" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A37" s="8" t="s">
         <v>14</v>
       </c>
@@ -2527,7 +2528,7 @@
       <c r="D37" s="10"/>
       <c r="E37" s="11"/>
     </row>
-    <row r="38" spans="1:5" ht="24" customHeight="1">
+    <row r="38" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A38" s="8" t="s">
         <v>10</v>
       </c>
@@ -2540,7 +2541,7 @@
       <c r="D38" s="10"/>
       <c r="E38" s="11"/>
     </row>
-    <row r="39" spans="1:5" ht="24" customHeight="1">
+    <row r="39" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A39" s="8" t="s">
         <v>14</v>
       </c>
@@ -2553,7 +2554,7 @@
       <c r="D39" s="10"/>
       <c r="E39" s="11"/>
     </row>
-    <row r="40" spans="1:5" ht="24" customHeight="1">
+    <row r="40" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A40" s="8" t="s">
         <v>10</v>
       </c>
@@ -2566,7 +2567,7 @@
       <c r="D40" s="10"/>
       <c r="E40" s="11"/>
     </row>
-    <row r="41" spans="1:5" ht="24" customHeight="1">
+    <row r="41" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A41" s="8" t="s">
         <v>14</v>
       </c>
@@ -2637,7 +2638,7 @@
       </c>
       <c r="E45" s="11"/>
     </row>
-    <row r="46" spans="1:5" ht="24" customHeight="1">
+    <row r="46" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A46" s="12">
         <v>600</v>
       </c>
@@ -2652,7 +2653,7 @@
       </c>
       <c r="E46" s="11"/>
     </row>
-    <row r="47" spans="1:5" ht="24" customHeight="1">
+    <row r="47" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A47" s="8" t="s">
         <v>14</v>
       </c>
@@ -2665,7 +2666,7 @@
       <c r="D47" s="10"/>
       <c r="E47" s="11"/>
     </row>
-    <row r="48" spans="1:5" ht="24" customHeight="1">
+    <row r="48" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A48" s="8" t="s">
         <v>10</v>
       </c>
@@ -2680,7 +2681,7 @@
       </c>
       <c r="E48" s="11"/>
     </row>
-    <row r="49" spans="1:5" ht="24" customHeight="1">
+    <row r="49" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A49" s="8" t="s">
         <v>10</v>
       </c>
@@ -2693,7 +2694,7 @@
       <c r="D49" s="10"/>
       <c r="E49" s="11"/>
     </row>
-    <row r="50" spans="1:5" ht="24" customHeight="1">
+    <row r="50" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A50" s="8" t="s">
         <v>10</v>
       </c>
@@ -2706,7 +2707,7 @@
       <c r="D50" s="10"/>
       <c r="E50" s="11"/>
     </row>
-    <row r="51" spans="1:5" ht="24" customHeight="1">
+    <row r="51" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A51" s="8" t="s">
         <v>10</v>
       </c>
@@ -2719,7 +2720,7 @@
       <c r="D51" s="10"/>
       <c r="E51" s="11"/>
     </row>
-    <row r="52" spans="1:5" ht="24" customHeight="1">
+    <row r="52" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A52" s="12">
         <v>600</v>
       </c>
@@ -2734,7 +2735,7 @@
       </c>
       <c r="E52" s="11"/>
     </row>
-    <row r="53" spans="1:5" ht="24" customHeight="1">
+    <row r="53" spans="1:5" ht="30">
       <c r="A53" s="8" t="s">
         <v>10</v>
       </c>
@@ -2818,7 +2819,7 @@
       </c>
       <c r="E58" s="11"/>
     </row>
-    <row r="59" spans="1:5" ht="24" customHeight="1">
+    <row r="59" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A59" s="8" t="s">
         <v>10</v>
       </c>
@@ -2833,7 +2834,7 @@
       </c>
       <c r="E59" s="11"/>
     </row>
-    <row r="60" spans="1:5" ht="24" customHeight="1">
+    <row r="60" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A60" s="8" t="s">
         <v>10</v>
       </c>
@@ -2888,7 +2889,7 @@
       </c>
       <c r="E63" s="11"/>
     </row>
-    <row r="64" spans="1:5" ht="24" customHeight="1">
+    <row r="64" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A64" s="8" t="s">
         <v>10</v>
       </c>
@@ -2901,7 +2902,7 @@
       <c r="D64" s="10"/>
       <c r="E64" s="11"/>
     </row>
-    <row r="65" spans="1:5" ht="24" customHeight="1">
+    <row r="65" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A65" s="8" t="s">
         <v>10</v>
       </c>
@@ -2914,7 +2915,7 @@
       <c r="D65" s="10"/>
       <c r="E65" s="11"/>
     </row>
-    <row r="66" spans="1:5" ht="24" customHeight="1">
+    <row r="66" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A66" s="8" t="s">
         <v>10</v>
       </c>
@@ -2927,7 +2928,7 @@
       <c r="D66" s="10"/>
       <c r="E66" s="11"/>
     </row>
-    <row r="67" spans="1:5" ht="24" customHeight="1">
+    <row r="67" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A67" s="8" t="s">
         <v>10</v>
       </c>
@@ -2942,7 +2943,7 @@
       </c>
       <c r="E67" s="11"/>
     </row>
-    <row r="68" spans="1:5" ht="24" customHeight="1">
+    <row r="68" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A68" s="8" t="s">
         <v>10</v>
       </c>
@@ -2955,7 +2956,7 @@
       <c r="D68" s="10"/>
       <c r="E68" s="11"/>
     </row>
-    <row r="69" spans="1:5" ht="24" customHeight="1">
+    <row r="69" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A69" s="8" t="s">
         <v>10</v>
       </c>
@@ -2968,7 +2969,7 @@
       <c r="D69" s="10"/>
       <c r="E69" s="11"/>
     </row>
-    <row r="70" spans="1:5" ht="24" customHeight="1">
+    <row r="70" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A70" s="8" t="s">
         <v>10</v>
       </c>
@@ -2983,7 +2984,7 @@
       </c>
       <c r="E70" s="11"/>
     </row>
-    <row r="71" spans="1:5" ht="24" customHeight="1">
+    <row r="71" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A71" s="8" t="s">
         <v>14</v>
       </c>
@@ -2996,7 +2997,7 @@
       <c r="D71" s="10"/>
       <c r="E71" s="11"/>
     </row>
-    <row r="72" spans="1:5" ht="24" customHeight="1">
+    <row r="72" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A72" s="8" t="s">
         <v>14</v>
       </c>
@@ -3009,7 +3010,7 @@
       <c r="D72" s="10"/>
       <c r="E72" s="11"/>
     </row>
-    <row r="73" spans="1:5" ht="24" customHeight="1">
+    <row r="73" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A73" s="8" t="s">
         <v>10</v>
       </c>
@@ -3022,7 +3023,7 @@
       <c r="D73" s="10"/>
       <c r="E73" s="11"/>
     </row>
-    <row r="74" spans="1:5" ht="24" customHeight="1">
+    <row r="74" spans="1:5" ht="24" hidden="1" customHeight="1">
       <c r="A74" s="8" t="s">
         <v>10</v>
       </c>
@@ -3932,7 +3933,13 @@
       <c r="E200" s="13"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:A200" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
+  <autoFilter ref="A1:D76" xr:uid="{00000000-0001-0000-0100-000000000000}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="超充电状态"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <phoneticPr fontId="8" type="noConversion"/>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A200" xr:uid="{00000000-0002-0000-0100-000000000000}">

</xml_diff>